<commit_message>
Remove Excel temp file; update workbook
Delete the Excel temporary/lock file (~$... .xlsx) and commit an updated binary .xlsx workbook. Cleans up the stray temp file and records the changed workbook content.
</commit_message>
<xml_diff>
--- a/選択項目マスタ.xlsx
+++ b/選択項目マスタ.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hirokishiga/Documents/development/ccta-repo-input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69846EE4-4F17-ED40-9439-5B333CDD3E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12198904-972C-E544-BEBC-BF668FF20CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="540" yWindow="660" windowWidth="13960" windowHeight="17260" xr2:uid="{B6DD94FA-2367-C94B-B0C5-1A336C551918}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="冠動脈" sheetId="1" r:id="rId1"/>
+    <sheet name="バイパス" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="55">
   <si>
     <t>血管</t>
     <rPh sb="0" eb="2">
@@ -252,6 +253,68 @@
   </si>
   <si>
     <t>Spotty calcification</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>LITA-</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>RITA-</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ao-SVG-</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ao-RA-</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ao-GEA-</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>評価</t>
+    <rPh sb="0" eb="2">
+      <t xml:space="preserve">ヒョウカ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>グラフト起始部〜吻合部において、明らかな有意狭窄所見を認めません。吻合部以遠の血流も</t>
+    <rPh sb="4" eb="7">
+      <t xml:space="preserve">キシブ </t>
+    </rPh>
+    <rPh sb="8" eb="11">
+      <t xml:space="preserve">フンゴウブ </t>
+    </rPh>
+    <rPh sb="16" eb="17">
+      <t xml:space="preserve">アキラカナ </t>
+    </rPh>
+    <rPh sb="20" eb="24">
+      <t xml:space="preserve">ユウイキョウサク </t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t xml:space="preserve">ショケン </t>
+    </rPh>
+    <rPh sb="27" eb="28">
+      <t xml:space="preserve">ミトメマセン </t>
+    </rPh>
+    <rPh sb="33" eb="36">
+      <t xml:space="preserve">フンゴウブイエンノ </t>
+    </rPh>
+    <rPh sb="36" eb="38">
+      <t xml:space="preserve">イエン </t>
+    </rPh>
+    <rPh sb="39" eb="41">
+      <t xml:space="preserve">ケツリュウモ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>small</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -813,6 +876,9 @@
       <c r="B12" t="s">
         <v>20</v>
       </c>
+      <c r="D12" s="2" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="13" spans="1:6">
       <c r="B13" t="s">
@@ -847,6 +913,53 @@
     <row r="19" spans="2:2">
       <c r="B19" t="s">
         <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10E2226E-3E49-0A4A-8404-9C499F9D8870}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>